<commit_message>
Combined scan results 2026-09-29
</commit_message>
<xml_diff>
--- a/results/2026-09-29.xlsx
+++ b/results/2026-09-29.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,18 +457,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>ABCL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>AAPL</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NTES</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>AAON</t>
@@ -482,26 +486,30 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AEHR</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REG</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>ACLS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>AMRX</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ALAB</t>
         </is>
       </c>
     </row>
@@ -514,13 +522,13 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>ARQT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>ALNT</t>
         </is>
       </c>
     </row>
@@ -528,18 +536,18 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CAMT</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>ARW</t>
         </is>
       </c>
     </row>
@@ -547,18 +555,18 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>CRUS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ALNT</t>
+          <t>BATRK</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>AVO</t>
         </is>
       </c>
     </row>
@@ -566,18 +574,18 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CRUS</t>
+          <t>ENSG</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>BIIB</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FEIM</t>
+          <t>AVT</t>
         </is>
       </c>
     </row>
@@ -585,18 +593,18 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BLFS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>IDCC</t>
+          <t>BAND</t>
         </is>
       </c>
     </row>
@@ -604,18 +612,18 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>HON</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ARW</t>
+          <t>BRKR</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>COHU</t>
         </is>
       </c>
     </row>
@@ -623,18 +631,18 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AVO</t>
+          <t>CDNA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>CROX</t>
         </is>
       </c>
     </row>
@@ -642,18 +650,18 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>LUNR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>CRWD</t>
         </is>
       </c>
     </row>
@@ -661,18 +669,18 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>NVMI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AXTI</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>DGII</t>
         </is>
       </c>
     </row>
@@ -680,18 +688,18 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LUNR</t>
+          <t>NVTS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BAND</t>
+          <t>GRAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>DIOD</t>
         </is>
       </c>
     </row>
@@ -699,18 +707,18 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MCHP</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BATRK</t>
+          <t>ILMN</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>DXPE</t>
         </is>
       </c>
     </row>
@@ -718,18 +726,18 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NVTS</t>
+          <t>ORLY</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>EMBJ</t>
         </is>
       </c>
     </row>
@@ -737,409 +745,413 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BLFS</t>
+          <t>KOD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>OMER</t>
+          <t>ENTG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>RYAAY</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BRKR</t>
+          <t>LGND</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PGEN</t>
+          <t>ETON</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SHMD</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>EXEL</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COHU</t>
+          <t>LTRX</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FAST</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>MAR</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FORM</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NDSN</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>GH</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DGII</t>
+          <t>NNBR</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>IRDM</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DIOD</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>MPWR</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DXPE</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>EMBJ</t>
+          <t>ONC</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>ORIC</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>MTSI</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>OUST</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>MXL</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>PENG</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>QMCO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>PGEN</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>RGEN</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IRDM</t>
+          <t>SATL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>PLXS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>SITM</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
-          <t>KOPN</t>
+          <t>SONO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PRTH</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>SRZN</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>SANM</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LTRX</t>
+          <t>VSXY</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>SIMO</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>MPWR</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>MRNA</t>
-        </is>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>STX</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>MTSI</t>
-        </is>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>VICR</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>MXL</t>
-        </is>
-      </c>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>XMTR</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>NDSN</t>
-        </is>
-      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>NNBR</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>NTAP</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>NTRA</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>OPRT</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ORIC</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>OUST</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>PENG</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>XNCR</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1152,7 +1164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1180,394 +1192,146 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AEHR</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PENG</t>
+          <t>CAI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GOOGN</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>GMAB</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>ISRG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>QMCO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CRSP</t>
+          <t>P</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CIFR</t>
+          <t>NTAP</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>KEEL</t>
+          <t>MXL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GLXY</t>
+          <t>SDGR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GMAB</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>EMBJ</t>
-        </is>
-      </c>
+          <t>QUBT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GOOG</t>
+          <t>USDE</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CBRS</t>
+          <t>STRC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IREN</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ENTG</t>
-        </is>
-      </c>
+          <t>OUST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>MRNA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>SECZ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>OUST</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>EXEL</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>DDOG</t>
-        </is>
-      </c>
+          <t>ILMN</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>QMCO</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GLBE</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>RKLB</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>BRKR</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SMCI</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>LITE</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>AXTI</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>CLSK</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>NTRA</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
           <t>GLND</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>CRWD</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>INOD</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>SONO</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>CYPH</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MDB</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>TECH</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>MXL</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>FAST</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>MU</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>BAND</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>NEOG</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>FIVN</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>PANW</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>GRML</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>PGEN</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>GH</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SMTC</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>AMRX</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>QCOM</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>HOOD</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TER</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>STX</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>USDE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>HUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>BETA</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>FPS</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>IOVA</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>INFQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>INTC</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>MRNA</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>ISRG</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>